<commit_message>
updating keen with v 2.0 fields
</commit_message>
<xml_diff>
--- a/KEEN 30m Subtidal Example/GOOS_EOV_Administrative_Info.xlsx
+++ b/KEEN 30m Subtidal Example/GOOS_EOV_Administrative_Info.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jebyrnes/Library/CloudStorage/GoogleDrive-jarrett.byrnes@gmail.com/.shortcut-targets-by-id/1uNfJ83WmlmCErHo4iUjWr1UYx8ZEmsih/Macroalgal EOV Data Processing docs/SOP_Visual/goos_data_sheets_and_entry_forms/KEEN 30m Subtidal Example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3D405B-7564-B848-800D-A4949C020A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D2830B-1B64-8045-8E1B-638A84B6365A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="1220" windowWidth="27640" windowHeight="16940" xr2:uid="{3BB4A0A6-1544-394D-83A2-653BD8DB631A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="Dataset Info" sheetId="4" r:id="rId1"/>
     <sheet name="Organization Info" sheetId="1" r:id="rId2"/>
     <sheet name="Observer Info" sheetId="3" r:id="rId3"/>
     <sheet name="Metadata" sheetId="2" r:id="rId4"/>

</xml_diff>